<commit_message>
fix: admin responsiveness, payos pending filter and excel styling
</commit_message>
<xml_diff>
--- a/Fake_data_template_v2.xlsx
+++ b/Fake_data_template_v2.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3420A651-C736-4417-931E-5A0737F1CDC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED1886AD-0972-49C4-9318-CE0153043730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2652" yWindow="2652" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Seed Data Form" sheetId="1" r:id="rId1"/>
@@ -516,7 +516,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B2" t="s">
@@ -566,6 +566,7 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="I2" r:id="rId1" xr:uid="{C62DEBE0-5CFB-4CF2-9C62-19CC4C5DBADD}"/>
+    <hyperlink ref="A2" r:id="rId2" xr:uid="{A96FDE0B-E79F-415B-AAD0-EB54FB6F003C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>